<commit_message>
Thêm trường MALOP cho File
</commit_message>
<xml_diff>
--- a/BlueSchoolSystem/DATA/SinhVien.xlsx
+++ b/BlueSchoolSystem/DATA/SinhVien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tai Lieu Hoc Tap\Do An Chuyen Nganh\BlueSchoolSystem\BlueSchoolSystem\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15928DBE-7B5D-4803-8B47-3C5188C47F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FC261C-B233-46CE-A76E-CCD76E490E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5B7985DB-BA14-4DE4-A325-153B5840A582}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="427" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="309">
   <si>
     <t>Mã số sinh viên</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Ngày tốt nghiệp dự kiến</t>
   </si>
   <si>
-    <t>Ghi chú</t>
-  </si>
-  <si>
     <t>2280604506</t>
   </si>
   <si>
@@ -949,13 +946,19 @@
   </si>
   <si>
     <t>HCM</t>
+  </si>
+  <si>
+    <t>Mã lớp</t>
+  </si>
+  <si>
+    <t>22DTHG1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -974,6 +977,12 @@
     <font>
       <sz val="14"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="163"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
@@ -1381,7 +1390,7 @@
     <col min="9" max="9" width="8.08984375" style="2" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="16.1796875" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="25.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.54296875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="16384" width="8.7265625" style="2"/>
   </cols>
   <sheetData>
@@ -1420,526 +1429,568 @@
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>307</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B2" s="10">
         <v>942040092421</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J2" s="9">
         <v>45890</v>
       </c>
       <c r="K2" s="9">
         <v>47351</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" s="10">
         <v>942040092422</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J3" s="9">
         <v>45890</v>
       </c>
       <c r="K3" s="9">
         <v>47351</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="10">
         <v>942040092424</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J4" s="9">
         <v>45890</v>
       </c>
       <c r="K4" s="9">
         <v>47351</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B5" s="10">
         <v>942040092425.33301</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J5" s="9">
         <v>45890</v>
       </c>
       <c r="K5" s="9">
         <v>47351</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" s="10">
         <v>942040092426.83301</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J6" s="9">
         <v>45890</v>
       </c>
       <c r="K6" s="9">
         <v>47351</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="10">
         <v>942040092428.33301</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J7" s="9">
         <v>45890</v>
       </c>
       <c r="K7" s="9">
         <v>47351</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" s="10">
         <v>942040092429.83301</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J8" s="9">
         <v>45890</v>
       </c>
       <c r="K8" s="9">
         <v>47351</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" s="10">
         <v>942040092431.33301</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J9" s="9">
         <v>45890</v>
       </c>
       <c r="K9" s="9">
         <v>47351</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B10" s="10">
         <v>942040092432.83301</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J10" s="9">
         <v>45890</v>
       </c>
       <c r="K10" s="9">
         <v>47351</v>
+      </c>
+      <c r="L10" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" s="10">
         <v>942040092434.33301</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J11" s="9">
         <v>45890</v>
       </c>
       <c r="K11" s="9">
         <v>47351</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B12" s="10">
         <v>942040092435.83301</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J12" s="9">
         <v>45890</v>
       </c>
       <c r="K12" s="9">
         <v>47351</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B13" s="10">
         <v>942040092437.33301</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J13" s="9">
         <v>45890</v>
       </c>
       <c r="K13" s="9">
         <v>47351</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="10">
         <v>942040092438.83301</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J14" s="9">
         <v>45890</v>
       </c>
       <c r="K14" s="9">
         <v>47351</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B15" s="10">
         <v>942040092440.33301</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J15" s="9">
         <v>45890</v>
       </c>
       <c r="K15" s="9">
         <v>47351</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>308</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B16" s="10">
         <v>942040092441.83301</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J16" s="9">
         <v>45890</v>
@@ -1947,34 +1998,37 @@
       <c r="K16" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L16" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B17" s="10">
         <v>942040092443.33301</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J17" s="9">
         <v>45890</v>
@@ -1982,34 +2036,37 @@
       <c r="K17" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L17" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B18" s="10">
         <v>942040092444.83301</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J18" s="9">
         <v>45890</v>
@@ -2017,34 +2074,37 @@
       <c r="K18" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L18" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B19" s="10">
         <v>942040092446.33301</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J19" s="9">
         <v>45890</v>
@@ -2052,34 +2112,37 @@
       <c r="K19" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L19" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B20" s="10">
         <v>942040092447.83301</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J20" s="9">
         <v>45890</v>
@@ -2087,34 +2150,37 @@
       <c r="K20" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L20" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B21" s="10">
         <v>942040092449.33301</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J21" s="9">
         <v>45890</v>
@@ -2122,34 +2188,37 @@
       <c r="K21" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L21" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22" s="10">
         <v>942040092450.83301</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J22" s="9">
         <v>45890</v>
@@ -2157,34 +2226,37 @@
       <c r="K22" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L22" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B23" s="10">
         <v>942040092452.33301</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J23" s="9">
         <v>45890</v>
@@ -2192,34 +2264,37 @@
       <c r="K23" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L23" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B24" s="10">
         <v>942040092453.83301</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J24" s="9">
         <v>45890</v>
@@ -2227,34 +2302,37 @@
       <c r="K24" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L24" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B25" s="10">
         <v>942040092455.33301</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J25" s="9">
         <v>45890</v>
@@ -2262,34 +2340,37 @@
       <c r="K25" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L25" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B26" s="10">
         <v>942040092456.83301</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J26" s="9">
         <v>45890</v>
@@ -2297,34 +2378,37 @@
       <c r="K26" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L26" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B27" s="10">
         <v>942040092458.33301</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J27" s="9">
         <v>45890</v>
@@ -2332,34 +2416,37 @@
       <c r="K27" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L27" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B28" s="10">
         <v>942040092459.83301</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J28" s="9">
         <v>45890</v>
@@ -2367,34 +2454,37 @@
       <c r="K28" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L28" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B29" s="10">
         <v>942040092461.33301</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J29" s="9">
         <v>45890</v>
@@ -2402,34 +2492,37 @@
       <c r="K29" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L29" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B30" s="10">
         <v>942040092462.83301</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J30" s="9">
         <v>45890</v>
@@ -2437,34 +2530,37 @@
       <c r="K30" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L30" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31" s="10">
         <v>942040092464.33301</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J31" s="9">
         <v>45890</v>
@@ -2472,34 +2568,37 @@
       <c r="K31" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L31" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B32" s="10">
         <v>942040092465.83301</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J32" s="9">
         <v>45890</v>
@@ -2507,34 +2606,37 @@
       <c r="K32" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L32" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B33" s="10">
         <v>942040092467.33301</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J33" s="9">
         <v>45890</v>
@@ -2542,34 +2644,37 @@
       <c r="K33" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L33" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B34" s="10">
         <v>942040092468.83301</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J34" s="9">
         <v>45890</v>
@@ -2577,34 +2682,37 @@
       <c r="K34" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L34" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B35" s="10">
         <v>942040092470.33301</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J35" s="9">
         <v>45890</v>
@@ -2612,8 +2720,11 @@
       <c r="K35" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L35" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A36" s="4">
         <v>2280602393</v>
       </c>
@@ -2621,25 +2732,25 @@
         <v>942040092471.83301</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J36" s="9">
         <v>45890</v>
@@ -2647,34 +2758,37 @@
       <c r="K36" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L36" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B37" s="10">
         <v>942040092473.33301</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J37" s="9">
         <v>45890</v>
@@ -2682,34 +2796,37 @@
       <c r="K37" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L37" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B38" s="10">
         <v>942040092474.83301</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J38" s="9">
         <v>45890</v>
@@ -2717,34 +2834,37 @@
       <c r="K38" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L38" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B39" s="10">
         <v>942040092476.33301</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J39" s="9">
         <v>45890</v>
@@ -2752,34 +2872,37 @@
       <c r="K39" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L39" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B40" s="10">
         <v>942040092477.83301</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J40" s="9">
         <v>45890</v>
@@ -2787,34 +2910,37 @@
       <c r="K40" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L40" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B41" s="10">
         <v>942040092479.33301</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J41" s="9">
         <v>45890</v>
@@ -2822,34 +2948,37 @@
       <c r="K41" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L41" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B42" s="10">
         <v>942040092480.83301</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J42" s="9">
         <v>45890</v>
@@ -2857,34 +2986,37 @@
       <c r="K42" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L42" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B43" s="10">
         <v>942040092482.33301</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J43" s="9">
         <v>45890</v>
@@ -2892,34 +3024,37 @@
       <c r="K43" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L43" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B44" s="10">
         <v>942040092483.83301</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J44" s="9">
         <v>45890</v>
@@ -2927,34 +3062,37 @@
       <c r="K44" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L44" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B45" s="10">
         <v>942040092485.33301</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J45" s="9">
         <v>45890</v>
@@ -2962,34 +3100,37 @@
       <c r="K45" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L45" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B46" s="10">
         <v>942040092486.83301</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J46" s="9">
         <v>45890</v>
@@ -2997,34 +3138,37 @@
       <c r="K46" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L46" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B47" s="10">
         <v>942040092488.33301</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J47" s="9">
         <v>45890</v>
@@ -3032,34 +3176,37 @@
       <c r="K47" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L47" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B48" s="10">
         <v>942040092489.83301</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J48" s="9">
         <v>45890</v>
@@ -3067,34 +3214,37 @@
       <c r="K48" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L48" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B49" s="10">
         <v>942040092491.33301</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="H49" s="8" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J49" s="9">
         <v>45890</v>
@@ -3102,34 +3252,37 @@
       <c r="K49" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L49" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B50" s="10">
         <v>942040092492.83301</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J50" s="9">
         <v>45890</v>
@@ -3137,34 +3290,37 @@
       <c r="K50" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L50" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B51" s="10">
         <v>942040092494.33301</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="H51" s="8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J51" s="9">
         <v>45890</v>
@@ -3172,34 +3328,37 @@
       <c r="K51" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L51" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B52" s="10">
         <v>942040092495.83301</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="F52" s="3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="G52" s="8" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="H52" s="8" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J52" s="9">
         <v>45890</v>
@@ -3207,34 +3366,37 @@
       <c r="K52" s="9">
         <v>47351</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L52" s="2" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B53" s="10">
         <v>942040092497.33301</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D53" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E53" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G53" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H53" s="8" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J53" s="9">
         <v>45890</v>
@@ -3242,8 +3404,12 @@
       <c r="K53" s="9">
         <v>47351</v>
       </c>
+      <c r="L53" s="2" t="s">
+        <v>308</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Cập nhật dữ liệu mẫu Sinh Viên
</commit_message>
<xml_diff>
--- a/BlueSchoolSystem/DATA/SinhVien.xlsx
+++ b/BlueSchoolSystem/DATA/SinhVien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tai Lieu Hoc Tap\Do An Chuyen Nganh\BlueSchoolSystem\BlueSchoolSystem\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FC261C-B233-46CE-A76E-CCD76E490E31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013DFB92-FB14-4B4F-A243-585AEE04A1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5B7985DB-BA14-4DE4-A325-153B5840A582}"/>
   </bookViews>
@@ -1461,10 +1461,10 @@
         <v>306</v>
       </c>
       <c r="J2" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K2" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>308</v>
@@ -1499,10 +1499,10 @@
         <v>306</v>
       </c>
       <c r="J3" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K3" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>308</v>
@@ -1537,10 +1537,10 @@
         <v>306</v>
       </c>
       <c r="J4" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K4" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>308</v>
@@ -1575,10 +1575,10 @@
         <v>306</v>
       </c>
       <c r="J5" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K5" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>308</v>
@@ -1613,10 +1613,10 @@
         <v>306</v>
       </c>
       <c r="J6" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K6" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>308</v>
@@ -1651,10 +1651,10 @@
         <v>306</v>
       </c>
       <c r="J7" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K7" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>308</v>
@@ -1689,10 +1689,10 @@
         <v>306</v>
       </c>
       <c r="J8" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K8" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>308</v>
@@ -1727,10 +1727,10 @@
         <v>306</v>
       </c>
       <c r="J9" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K9" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>308</v>
@@ -1765,10 +1765,10 @@
         <v>306</v>
       </c>
       <c r="J10" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K10" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>308</v>
@@ -1803,10 +1803,10 @@
         <v>306</v>
       </c>
       <c r="J11" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K11" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>308</v>
@@ -1841,10 +1841,10 @@
         <v>306</v>
       </c>
       <c r="J12" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K12" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>308</v>
@@ -1879,10 +1879,10 @@
         <v>306</v>
       </c>
       <c r="J13" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K13" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>308</v>
@@ -1917,10 +1917,10 @@
         <v>306</v>
       </c>
       <c r="J14" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K14" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L14" s="2" t="s">
         <v>308</v>
@@ -1955,10 +1955,10 @@
         <v>306</v>
       </c>
       <c r="J15" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K15" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>308</v>
@@ -1993,10 +1993,10 @@
         <v>306</v>
       </c>
       <c r="J16" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K16" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>308</v>
@@ -2031,10 +2031,10 @@
         <v>306</v>
       </c>
       <c r="J17" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K17" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>308</v>
@@ -2069,10 +2069,10 @@
         <v>306</v>
       </c>
       <c r="J18" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K18" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>308</v>
@@ -2107,10 +2107,10 @@
         <v>306</v>
       </c>
       <c r="J19" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K19" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>308</v>
@@ -2145,10 +2145,10 @@
         <v>306</v>
       </c>
       <c r="J20" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K20" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>308</v>
@@ -2183,10 +2183,10 @@
         <v>306</v>
       </c>
       <c r="J21" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K21" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>308</v>
@@ -2221,10 +2221,10 @@
         <v>306</v>
       </c>
       <c r="J22" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K22" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>308</v>
@@ -2259,10 +2259,10 @@
         <v>306</v>
       </c>
       <c r="J23" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K23" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>308</v>
@@ -2297,10 +2297,10 @@
         <v>306</v>
       </c>
       <c r="J24" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K24" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>308</v>
@@ -2335,10 +2335,10 @@
         <v>306</v>
       </c>
       <c r="J25" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K25" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L25" s="2" t="s">
         <v>308</v>
@@ -2373,10 +2373,10 @@
         <v>306</v>
       </c>
       <c r="J26" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K26" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>308</v>
@@ -2411,10 +2411,10 @@
         <v>306</v>
       </c>
       <c r="J27" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K27" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>308</v>
@@ -2449,10 +2449,10 @@
         <v>306</v>
       </c>
       <c r="J28" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K28" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>308</v>
@@ -2487,10 +2487,10 @@
         <v>306</v>
       </c>
       <c r="J29" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K29" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>308</v>
@@ -2525,10 +2525,10 @@
         <v>306</v>
       </c>
       <c r="J30" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K30" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>308</v>
@@ -2563,10 +2563,10 @@
         <v>306</v>
       </c>
       <c r="J31" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K31" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L31" s="2" t="s">
         <v>308</v>
@@ -2601,10 +2601,10 @@
         <v>306</v>
       </c>
       <c r="J32" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K32" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>308</v>
@@ -2639,10 +2639,10 @@
         <v>306</v>
       </c>
       <c r="J33" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K33" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>308</v>
@@ -2677,10 +2677,10 @@
         <v>306</v>
       </c>
       <c r="J34" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K34" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L34" s="2" t="s">
         <v>308</v>
@@ -2715,10 +2715,10 @@
         <v>306</v>
       </c>
       <c r="J35" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K35" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L35" s="2" t="s">
         <v>308</v>
@@ -2753,10 +2753,10 @@
         <v>306</v>
       </c>
       <c r="J36" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K36" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>308</v>
@@ -2791,10 +2791,10 @@
         <v>306</v>
       </c>
       <c r="J37" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K37" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L37" s="2" t="s">
         <v>308</v>
@@ -2829,10 +2829,10 @@
         <v>306</v>
       </c>
       <c r="J38" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K38" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L38" s="2" t="s">
         <v>308</v>
@@ -2867,10 +2867,10 @@
         <v>306</v>
       </c>
       <c r="J39" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K39" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L39" s="2" t="s">
         <v>308</v>
@@ -2905,10 +2905,10 @@
         <v>306</v>
       </c>
       <c r="J40" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K40" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L40" s="2" t="s">
         <v>308</v>
@@ -2943,10 +2943,10 @@
         <v>306</v>
       </c>
       <c r="J41" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K41" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>308</v>
@@ -2981,10 +2981,10 @@
         <v>306</v>
       </c>
       <c r="J42" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K42" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>308</v>
@@ -3019,10 +3019,10 @@
         <v>306</v>
       </c>
       <c r="J43" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K43" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>308</v>
@@ -3057,10 +3057,10 @@
         <v>306</v>
       </c>
       <c r="J44" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K44" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>308</v>
@@ -3095,10 +3095,10 @@
         <v>306</v>
       </c>
       <c r="J45" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K45" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L45" s="2" t="s">
         <v>308</v>
@@ -3133,10 +3133,10 @@
         <v>306</v>
       </c>
       <c r="J46" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K46" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L46" s="2" t="s">
         <v>308</v>
@@ -3171,10 +3171,10 @@
         <v>306</v>
       </c>
       <c r="J47" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K47" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L47" s="2" t="s">
         <v>308</v>
@@ -3209,10 +3209,10 @@
         <v>306</v>
       </c>
       <c r="J48" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K48" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L48" s="2" t="s">
         <v>308</v>
@@ -3247,10 +3247,10 @@
         <v>306</v>
       </c>
       <c r="J49" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K49" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L49" s="2" t="s">
         <v>308</v>
@@ -3285,10 +3285,10 @@
         <v>306</v>
       </c>
       <c r="J50" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K50" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L50" s="2" t="s">
         <v>308</v>
@@ -3323,10 +3323,10 @@
         <v>306</v>
       </c>
       <c r="J51" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K51" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L51" s="2" t="s">
         <v>308</v>
@@ -3361,10 +3361,10 @@
         <v>306</v>
       </c>
       <c r="J52" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K52" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L52" s="2" t="s">
         <v>308</v>
@@ -3399,10 +3399,10 @@
         <v>306</v>
       </c>
       <c r="J53" s="9">
-        <v>45890</v>
+        <v>44794</v>
       </c>
       <c r="K53" s="9">
-        <v>47351</v>
+        <v>46255</v>
       </c>
       <c r="L53" s="2" t="s">
         <v>308</v>

</xml_diff>

<commit_message>
Cập nhật dữ liệu mẫu trong thư mục DATA
</commit_message>
<xml_diff>
--- a/BlueSchoolSystem/DATA/SinhVien.xlsx
+++ b/BlueSchoolSystem/DATA/SinhVien.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Tai Lieu Hoc Tap\Do An Chuyen Nganh\BlueSchoolSystem\BlueSchoolSystem\DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BlueSchoolSystem\BlueSchoolSystem\DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013DFB92-FB14-4B4F-A243-585AEE04A1EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{319C8CB1-F762-4AAF-A5DD-B729FBDF13B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5B7985DB-BA14-4DE4-A325-153B5840A582}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="479" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="298">
   <si>
     <t>Mã số sinh viên</t>
   </si>
@@ -204,12 +204,6 @@
     <t>2280617797</t>
   </si>
   <si>
-    <t>2280603730</t>
-  </si>
-  <si>
-    <t>2280603732</t>
-  </si>
-  <si>
     <t>2280603808</t>
   </si>
   <si>
@@ -330,9 +324,6 @@
     <t>Vinh</t>
   </si>
   <si>
-    <t>Vũ</t>
-  </si>
-  <si>
     <t>Ý</t>
   </si>
   <si>
@@ -474,12 +465,6 @@
     <t xml:space="preserve">Bùi Quang </t>
   </si>
   <si>
-    <t xml:space="preserve">Huỳnh Tuấn </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lê Duy </t>
-  </si>
-  <si>
     <t xml:space="preserve">Nguyễn Trần Thiên </t>
   </si>
   <si>
@@ -621,12 +606,6 @@
     <t>09/03/2000</t>
   </si>
   <si>
-    <t>28/03/2004</t>
-  </si>
-  <si>
-    <t>03/01/2004</t>
-  </si>
-  <si>
     <t>NAM</t>
   </si>
   <si>
@@ -780,12 +759,6 @@
     <t>0792133833</t>
   </si>
   <si>
-    <t>0909594687</t>
-  </si>
-  <si>
-    <t>0792128236</t>
-  </si>
-  <si>
     <t>0946263563</t>
   </si>
   <si>
@@ -934,12 +907,6 @@
   </si>
   <si>
     <t>quangvinh090300@gmail.com</t>
-  </si>
-  <si>
-    <t>tuanvu2832004@gmail.com</t>
-  </si>
-  <si>
-    <t>leduyvupro123@gmail.com</t>
   </si>
   <si>
     <t>ntrthieny@gmail.com</t>
@@ -1002,7 +969,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -1036,11 +1003,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1062,6 +1038,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1376,7 +1365,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4498B72-87E6-421E-AA91-74E1F7474ACA}">
-  <dimension ref="A1:L53"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" style="2" bestFit="1" customWidth="1"/>
@@ -1429,7 +1418,7 @@
         <v>10</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.3">
@@ -1440,25 +1429,25 @@
         <v>942040092421</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="H2" s="8" t="s">
-        <v>254</v>
+        <v>245</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J2" s="9">
         <v>44794</v>
@@ -1467,7 +1456,7 @@
         <v>46255</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.3">
@@ -1478,25 +1467,25 @@
         <v>942040092422</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>255</v>
+        <v>246</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J3" s="9">
         <v>44794</v>
@@ -1505,7 +1494,7 @@
         <v>46255</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.3">
@@ -1516,25 +1505,25 @@
         <v>942040092424</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>256</v>
+        <v>247</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J4" s="9">
         <v>44794</v>
@@ -1543,7 +1532,7 @@
         <v>46255</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.3">
@@ -1554,25 +1543,25 @@
         <v>942040092425.33301</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>257</v>
+        <v>248</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J5" s="9">
         <v>44794</v>
@@ -1581,7 +1570,7 @@
         <v>46255</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.3">
@@ -1592,25 +1581,25 @@
         <v>942040092426.83301</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>258</v>
+        <v>249</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J6" s="9">
         <v>44794</v>
@@ -1619,7 +1608,7 @@
         <v>46255</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.3">
@@ -1630,25 +1619,25 @@
         <v>942040092428.33301</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="F7" s="3" t="s">
+        <v>193</v>
+      </c>
+      <c r="G7" s="8" t="s">
         <v>200</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>207</v>
-      </c>
       <c r="H7" s="8" t="s">
-        <v>259</v>
+        <v>250</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J7" s="9">
         <v>44794</v>
@@ -1657,7 +1646,7 @@
         <v>46255</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.3">
@@ -1668,25 +1657,25 @@
         <v>942040092429.83301</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>260</v>
+        <v>251</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J8" s="9">
         <v>44794</v>
@@ -1695,7 +1684,7 @@
         <v>46255</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.3">
@@ -1706,25 +1695,25 @@
         <v>942040092431.33301</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>261</v>
+        <v>252</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J9" s="9">
         <v>44794</v>
@@ -1733,7 +1722,7 @@
         <v>46255</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.3">
@@ -1744,25 +1733,25 @@
         <v>942040092432.83301</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>262</v>
+        <v>253</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J10" s="9">
         <v>44794</v>
@@ -1771,7 +1760,7 @@
         <v>46255</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.3">
@@ -1782,25 +1771,25 @@
         <v>942040092434.33301</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="H11" s="8" t="s">
-        <v>263</v>
+        <v>254</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J11" s="9">
         <v>44794</v>
@@ -1809,7 +1798,7 @@
         <v>46255</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.3">
@@ -1820,25 +1809,25 @@
         <v>942040092435.83301</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>264</v>
+        <v>255</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J12" s="9">
         <v>44794</v>
@@ -1847,7 +1836,7 @@
         <v>46255</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.3">
@@ -1858,25 +1847,25 @@
         <v>942040092437.33301</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>265</v>
+        <v>256</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J13" s="9">
         <v>44794</v>
@@ -1885,7 +1874,7 @@
         <v>46255</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.3">
@@ -1896,25 +1885,25 @@
         <v>942040092438.83301</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>266</v>
+        <v>257</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J14" s="9">
         <v>44794</v>
@@ -1923,7 +1912,7 @@
         <v>46255</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.3">
@@ -1934,25 +1923,25 @@
         <v>942040092440.33301</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G15" s="8" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="H15" s="8" t="s">
-        <v>267</v>
+        <v>258</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J15" s="9">
         <v>44794</v>
@@ -1961,7 +1950,7 @@
         <v>46255</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.3">
@@ -1972,25 +1961,25 @@
         <v>942040092441.83301</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G16" s="8" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="H16" s="8" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J16" s="9">
         <v>44794</v>
@@ -1999,7 +1988,7 @@
         <v>46255</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.3">
@@ -2010,25 +1999,25 @@
         <v>942040092443.33301</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G17" s="8" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="H17" s="8" t="s">
-        <v>269</v>
+        <v>260</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J17" s="9">
         <v>44794</v>
@@ -2037,7 +2026,7 @@
         <v>46255</v>
       </c>
       <c r="L17" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.3">
@@ -2048,25 +2037,25 @@
         <v>942040092444.83301</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G18" s="8" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="H18" s="8" t="s">
-        <v>270</v>
+        <v>261</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J18" s="9">
         <v>44794</v>
@@ -2075,7 +2064,7 @@
         <v>46255</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.3">
@@ -2086,25 +2075,25 @@
         <v>942040092446.33301</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>271</v>
+        <v>262</v>
       </c>
       <c r="I19" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J19" s="9">
         <v>44794</v>
@@ -2113,7 +2102,7 @@
         <v>46255</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.3">
@@ -2124,25 +2113,25 @@
         <v>942040092447.83301</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>272</v>
+        <v>263</v>
       </c>
       <c r="I20" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J20" s="9">
         <v>44794</v>
@@ -2151,7 +2140,7 @@
         <v>46255</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.3">
@@ -2162,25 +2151,25 @@
         <v>942040092449.33301</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>273</v>
+        <v>264</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J21" s="9">
         <v>44794</v>
@@ -2189,7 +2178,7 @@
         <v>46255</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.3">
@@ -2200,25 +2189,25 @@
         <v>942040092450.83301</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J22" s="9">
         <v>44794</v>
@@ -2227,7 +2216,7 @@
         <v>46255</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.3">
@@ -2238,25 +2227,25 @@
         <v>942040092452.33301</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J23" s="9">
         <v>44794</v>
@@ -2265,7 +2254,7 @@
         <v>46255</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.3">
@@ -2276,25 +2265,25 @@
         <v>942040092453.83301</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J24" s="9">
         <v>44794</v>
@@ -2303,7 +2292,7 @@
         <v>46255</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.3">
@@ -2314,25 +2303,25 @@
         <v>942040092455.33301</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>277</v>
+        <v>268</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J25" s="9">
         <v>44794</v>
@@ -2341,7 +2330,7 @@
         <v>46255</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.3">
@@ -2352,25 +2341,25 @@
         <v>942040092456.83301</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>278</v>
+        <v>269</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J26" s="9">
         <v>44794</v>
@@ -2379,7 +2368,7 @@
         <v>46255</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.3">
@@ -2390,25 +2379,25 @@
         <v>942040092458.33301</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="H27" s="8" t="s">
-        <v>279</v>
+        <v>270</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J27" s="9">
         <v>44794</v>
@@ -2417,7 +2406,7 @@
         <v>46255</v>
       </c>
       <c r="L27" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.3">
@@ -2428,25 +2417,25 @@
         <v>942040092459.83301</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>280</v>
+        <v>271</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J28" s="9">
         <v>44794</v>
@@ -2455,7 +2444,7 @@
         <v>46255</v>
       </c>
       <c r="L28" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.3">
@@ -2466,25 +2455,25 @@
         <v>942040092461.33301</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>281</v>
+        <v>272</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J29" s="9">
         <v>44794</v>
@@ -2493,7 +2482,7 @@
         <v>46255</v>
       </c>
       <c r="L29" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.3">
@@ -2504,25 +2493,25 @@
         <v>942040092462.83301</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>282</v>
+        <v>273</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J30" s="9">
         <v>44794</v>
@@ -2531,7 +2520,7 @@
         <v>46255</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.3">
@@ -2542,25 +2531,25 @@
         <v>942040092464.33301</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="F31" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G31" s="8" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="H31" s="8" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J31" s="9">
         <v>44794</v>
@@ -2569,7 +2558,7 @@
         <v>46255</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.3">
@@ -2580,25 +2569,25 @@
         <v>942040092465.83301</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="F32" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G32" s="8" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="H32" s="8" t="s">
-        <v>284</v>
+        <v>275</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J32" s="9">
         <v>44794</v>
@@ -2607,7 +2596,7 @@
         <v>46255</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
@@ -2618,25 +2607,25 @@
         <v>942040092467.33301</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G33" s="8" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="H33" s="8" t="s">
-        <v>285</v>
+        <v>276</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J33" s="9">
         <v>44794</v>
@@ -2645,7 +2634,7 @@
         <v>46255</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
@@ -2656,25 +2645,25 @@
         <v>942040092468.83301</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="F34" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G34" s="8" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="H34" s="8" t="s">
-        <v>286</v>
+        <v>277</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J34" s="9">
         <v>44794</v>
@@ -2683,7 +2672,7 @@
         <v>46255</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
@@ -2694,25 +2683,25 @@
         <v>942040092470.33301</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="F35" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G35" s="8" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="H35" s="8" t="s">
-        <v>287</v>
+        <v>278</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J35" s="9">
         <v>44794</v>
@@ -2721,7 +2710,7 @@
         <v>46255</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
@@ -2732,25 +2721,25 @@
         <v>942040092471.83301</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="F36" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G36" s="8" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="H36" s="8" t="s">
-        <v>288</v>
+        <v>279</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J36" s="9">
         <v>44794</v>
@@ -2759,7 +2748,7 @@
         <v>46255</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
@@ -2770,25 +2759,25 @@
         <v>942040092473.33301</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G37" s="8" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="H37" s="8" t="s">
-        <v>289</v>
+        <v>280</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J37" s="9">
         <v>44794</v>
@@ -2797,7 +2786,7 @@
         <v>46255</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -2808,25 +2797,25 @@
         <v>942040092474.83301</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="H38" s="8" t="s">
-        <v>290</v>
+        <v>281</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J38" s="9">
         <v>44794</v>
@@ -2835,7 +2824,7 @@
         <v>46255</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
@@ -2846,25 +2835,25 @@
         <v>942040092476.33301</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G39" s="8" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="H39" s="8" t="s">
-        <v>291</v>
+        <v>282</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J39" s="9">
         <v>44794</v>
@@ -2873,7 +2862,7 @@
         <v>46255</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
@@ -2884,25 +2873,25 @@
         <v>942040092477.83301</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="F40" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>240</v>
+        <v>233</v>
       </c>
       <c r="H40" s="8" t="s">
-        <v>292</v>
+        <v>283</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J40" s="9">
         <v>44794</v>
@@ -2911,7 +2900,7 @@
         <v>46255</v>
       </c>
       <c r="L40" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
@@ -2922,25 +2911,25 @@
         <v>942040092479.33301</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G41" s="8" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="H41" s="8" t="s">
-        <v>293</v>
+        <v>284</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J41" s="9">
         <v>44794</v>
@@ -2949,7 +2938,7 @@
         <v>46255</v>
       </c>
       <c r="L41" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
@@ -2960,25 +2949,25 @@
         <v>942040092480.83301</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="F42" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G42" s="8" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="H42" s="8" t="s">
-        <v>294</v>
+        <v>285</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J42" s="9">
         <v>44794</v>
@@ -2987,7 +2976,7 @@
         <v>46255</v>
       </c>
       <c r="L42" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
@@ -2998,25 +2987,25 @@
         <v>942040092482.33301</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G43" s="8" t="s">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="H43" s="8" t="s">
-        <v>295</v>
+        <v>286</v>
       </c>
       <c r="I43" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J43" s="9">
         <v>44794</v>
@@ -3025,7 +3014,7 @@
         <v>46255</v>
       </c>
       <c r="L43" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
@@ -3036,25 +3025,25 @@
         <v>942040092483.83301</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G44" s="8" t="s">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="H44" s="8" t="s">
-        <v>296</v>
+        <v>287</v>
       </c>
       <c r="I44" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J44" s="9">
         <v>44794</v>
@@ -3063,7 +3052,7 @@
         <v>46255</v>
       </c>
       <c r="L44" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.3">
@@ -3074,25 +3063,25 @@
         <v>942040092485.33301</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="F45" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G45" s="8" t="s">
-        <v>245</v>
+        <v>238</v>
       </c>
       <c r="H45" s="8" t="s">
-        <v>297</v>
+        <v>288</v>
       </c>
       <c r="I45" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J45" s="9">
         <v>44794</v>
@@ -3101,7 +3090,7 @@
         <v>46255</v>
       </c>
       <c r="L45" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.3">
@@ -3112,25 +3101,25 @@
         <v>942040092486.83301</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="G46" s="8" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="H46" s="8" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="I46" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J46" s="9">
         <v>44794</v>
@@ -3139,7 +3128,7 @@
         <v>46255</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
@@ -3150,25 +3139,25 @@
         <v>942040092488.33301</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D47" s="5" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G47" s="8" t="s">
-        <v>247</v>
+        <v>240</v>
       </c>
       <c r="H47" s="8" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="I47" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J47" s="9">
         <v>44794</v>
@@ -3177,7 +3166,7 @@
         <v>46255</v>
       </c>
       <c r="L47" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
@@ -3188,25 +3177,25 @@
         <v>942040092489.83301</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G48" s="8" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="H48" s="8" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="I48" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J48" s="9">
         <v>44794</v>
@@ -3215,7 +3204,7 @@
         <v>46255</v>
       </c>
       <c r="L48" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.3">
@@ -3226,25 +3215,25 @@
         <v>942040092491.33301</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="F49" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G49" s="8" t="s">
-        <v>249</v>
+        <v>242</v>
       </c>
       <c r="H49" s="8" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="I49" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J49" s="9">
         <v>44794</v>
@@ -3253,7 +3242,7 @@
         <v>46255</v>
       </c>
       <c r="L49" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
@@ -3264,25 +3253,25 @@
         <v>942040092492.83301</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="G50" s="8" t="s">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="H50" s="8" t="s">
-        <v>302</v>
+        <v>293</v>
       </c>
       <c r="I50" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J50" s="9">
         <v>44794</v>
@@ -3291,36 +3280,36 @@
         <v>46255</v>
       </c>
       <c r="L50" s="2" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B51" s="10">
-        <v>942040092494.33301</v>
+      <c r="B51" s="17">
+        <v>942040092497.33301</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E51" s="6" t="s">
-        <v>198</v>
+        <v>184</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>251</v>
+        <v>194</v>
+      </c>
+      <c r="G51" s="8" t="s">
+        <v>244</v>
       </c>
       <c r="H51" s="8" t="s">
-        <v>303</v>
+        <v>294</v>
       </c>
       <c r="I51" s="2" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="J51" s="9">
         <v>44794</v>
@@ -3329,84 +3318,18 @@
         <v>46255</v>
       </c>
       <c r="L51" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A52" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B52" s="10">
-        <v>942040092495.83301</v>
-      </c>
-      <c r="C52" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="D52" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="F52" s="3" t="s">
-        <v>200</v>
-      </c>
-      <c r="G52" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="H52" s="8" t="s">
-        <v>304</v>
-      </c>
-      <c r="I52" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="J52" s="9">
-        <v>44794</v>
-      </c>
-      <c r="K52" s="9">
-        <v>46255</v>
-      </c>
-      <c r="L52" s="2" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A53" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B53" s="10">
-        <v>942040092497.33301</v>
-      </c>
-      <c r="C53" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="D53" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="F53" s="3" t="s">
-        <v>201</v>
-      </c>
-      <c r="G53" s="8" t="s">
-        <v>253</v>
-      </c>
-      <c r="H53" s="8" t="s">
-        <v>305</v>
-      </c>
-      <c r="I53" s="2" t="s">
-        <v>306</v>
-      </c>
-      <c r="J53" s="9">
-        <v>44794</v>
-      </c>
-      <c r="K53" s="9">
-        <v>46255</v>
-      </c>
-      <c r="L53" s="2" t="s">
-        <v>308</v>
-      </c>
+        <v>297</v>
+      </c>
+    </row>
+    <row r="52" spans="1:12" s="14" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A52" s="13"/>
+      <c r="B52" s="15"/>
+      <c r="C52" s="11"/>
+      <c r="D52" s="11"/>
+      <c r="E52" s="12"/>
+      <c r="F52" s="13"/>
+      <c r="J52" s="16"/>
+      <c r="K52" s="16"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>